<commit_message>
Restore format_json_list in the hot-threat SQL and add a StarRocks twin UDF for the lab.
Co-authored-by: daydayup <removecode@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/业务SQL跑通记录.xlsx
+++ b/outputs/业务SQL跑通记录.xlsx
@@ -524,7 +524,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>已跑通：用户已确认。未记录：尚未登记最终 SQL，不表示一定没有跑通，也不表示跑不通。</t>
+          <t>已跑通：用户已确认。已跑通（改回UDF后待用户确认）：用户确认过的是旧写法，新写法只在本机执行过。未记录：尚未登记最终 SQL，不表示一定没有跑通，也不表示跑不通。</t>
         </is>
       </c>
     </row>
@@ -645,12 +645,12 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>已跑通</t>
+          <t>已跑通（改回UDF后待用户确认）</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>三条语句（黑域名、黑文件、黑 URL）均已跑通</t>
+          <t>三条语句此前用户确认已跑通；改回 UDF 写法后待用户确认</t>
         </is>
       </c>
     </row>
@@ -2233,7 +2233,7 @@
           get_json_object(str10_tmp, '$.info.attr') AS attr,
           str2 AS devid
    FROM csc.ods_csc_log_audit,
-        unnest(ifnull(cast(parse_json(regexp_replace(str10, '\\\\+"', '"')) AS ARRAY&lt;JSON&gt;), [])) AS str10_tbl(str10_tmp)
+        unnest(`default`.format_json_list(regexp_replace(str10, '\\\\+"', '"'))) AS str10_tbl(str10_tmp)
    WHERE app_id = 'analysis-proxy-api'
      AND module_id IN ('file_hash', 'file_scan')
      AND str1 IN ('VNGAF', 'NGAF', 'EDR', 'EDR_BOTNET', 'SIP', 'SIP_SMTP', 'SIP_SMB',
@@ -2252,7 +2252,7 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>已跑通</t>
+          <t>已跑通（改回UDF后待用户确认）</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -2262,12 +2262,12 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>用户确认已跑通（2026-10-16）。本机实验库另执行过三条：黑域名 110 行、黑文件 0 行、黑 URL 100 行（outputs/topthreat-hot-stat-results.tsv，ACT-042）。黑文件 0 行是本机造数的 long1 不为 0，不是语句报错。</t>
+          <t>用户确认已跑通的是 parse_json 写法（2026-10-16）。按 DEC-023 改回 format_json_list 后，只在本机 StarRocks 用 UDF 孪生实现执行过（ACT-046）：黑域名 320 行、黑文件 50 行、黑 URL 620 行，数据为合成数据。用户尚未在当前 StarRocks 确认改回后的语句。</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>库表改 csc.ods_csc_log_audit（DEC-014）；log_app_id 改 app_id（DEC-015）；explode(format_json_list()) 改 unnest(parse_json())（ACT-038）；加 SET_VAR(new_planner_optimize_timeout=60000)（DEC-022）。该语句没有 sodl 分支。旧 SQL 写死 day=20250826、hour=01，新语句写 day=20261001、hour=0（实验窗口）。</t>
+          <t>UDF 按 DEC-023 原样保留：`default`.format_json_list 包在 unnest 里，default 是保留字所以加反引号；ACT-038 的 parse_json 写法已撤回。库表改 csc.ods_csc_log_audit（DEC-014）；log_app_id 改 app_id（DEC-015）；explode(UDF) 改 unnest(UDF)；加 SET_VAR(new_planner_optimize_timeout=60000)（DEC-022）。该语句没有 sodl 分支。旧 SQL 写死 day=20250826、hour=01，新语句写 day=20261001、hour=0（实验窗口）。</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
      (SELECT lower(get_json_object(str10_tmp, '$.url')) AS url,
              str2 AS devid
       FROM csc.ods_csc_log_audit,
-           unnest(ifnull(cast(parse_json(regexp_replace(str10, '\\\\+"', '"')) AS ARRAY&lt;JSON&gt;), [])) AS str10_tbl(str10_tmp)
+           unnest(`default`.format_json_list(regexp_replace(str10, '\\\\+"', '"'))) AS str10_tbl(str10_tmp)
       WHERE app_id IN ('url-proxy-svc', 'cloudcheck')
         AND module_id IN ('url-proxy-svc', 'CloudCheck')
         AND str1 IN ('VNGAF', 'NGAF', 'EDR', 'EDR_BOTNET', 'SIP', 'SIP_SMTP', 'SIP_SMB',
@@ -2427,7 +2427,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>已跑通</t>
+          <t>已跑通（改回UDF后待用户确认）</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -2437,12 +2437,12 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>用户确认已跑通（2026-10-16）。本机实验库另执行过三条：黑域名 110 行、黑文件 0 行、黑 URL 100 行（outputs/topthreat-hot-stat-results.tsv，ACT-042）。黑文件 0 行是本机造数的 long1 不为 0，不是语句报错。</t>
+          <t>用户确认已跑通的是 parse_json 写法（2026-10-16）。按 DEC-023 改回 format_json_list 后，只在本机 StarRocks 用 UDF 孪生实现执行过（ACT-046）：黑域名 320 行、黑文件 50 行、黑 URL 620 行，数据为合成数据。用户尚未在当前 StarRocks 确认改回后的语句。</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>改写项同 black_domain_stat：库表、app_id、sodl 时间条件、count(1)、deviceId、unnest(parse_json())、规划超时提示；${day}/${hour} 写死为实验窗口 20261001 / 0。</t>
+          <t>UDF 按 DEC-023 原样保留：`default`.format_json_list 包在 unnest 里，default 是保留字所以加反引号；ACT-038 的 parse_json 写法已撤回。改写项同 black_domain_stat：库表、app_id、sodl 时间条件、count(1)、deviceId、unnest(UDF)、规划超时提示；${day}/${hour} 写死为实验窗口 20261001 / 0。</t>
         </is>
       </c>
     </row>
@@ -2567,7 +2567,7 @@
      (SELECT lower(get_json_object(str10_tmp, '$.domain')) AS domain,
              str2 AS devid
       FROM csc.ods_csc_log_audit,
-           unnest(ifnull(cast(parse_json(regexp_replace(str10, '\\\\+"', '"')) AS ARRAY&lt;JSON&gt;), [])) AS str10_tbl(str10_tmp)
+           unnest(`default`.format_json_list(regexp_replace(str10, '\\\\+"', '"'))) AS str10_tbl(str10_tmp)
       WHERE app_id IN ('domain-proxy-svc', 'cloudcheck')
         AND module_id IN ('domain-proxy-svc', 'CloudCheck')
         AND str1 IN ('VNGAF', 'NGAF', 'EDR', 'EDR_BOTNET', 'SIP', 'SIP_SMTP', 'SIP_SMB',
@@ -2613,7 +2613,7 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>已跑通</t>
+          <t>已跑通（改回UDF后待用户确认）</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -2623,12 +2623,12 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>用户确认已跑通（2026-10-16）。本机实验库另执行过三条：黑域名 110 行、黑文件 0 行、黑 URL 100 行（outputs/topthreat-hot-stat-results.tsv，ACT-042）。黑文件 0 行是本机造数的 long1 不为 0，不是语句报错。</t>
+          <t>用户确认已跑通的是 parse_json 写法（2026-10-16）。按 DEC-023 改回 format_json_list 后，只在本机 StarRocks 用 UDF 孪生实现执行过（ACT-046）：黑域名 320 行、黑文件 50 行、黑 URL 620 行，数据为合成数据。用户尚未在当前 StarRocks 确认改回后的语句。</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>库表 default.log_audit_source 改 csc.ods_csc_log_audit（DEC-014）；log_app_id 改 app_id（DEC-015）；sodl 的 day/hour 改 insertdate='2026-10-01' 与 hour(from_unixtime(inserttimestamp))=0（DEC-016/017）；sum(log_num) 改 count(1)（DEC-020）；MANAGE/manage 改 deviceId（DEC-021）；LATERAL VIEW explode(format_json_list()) 改 unnest(parse_json())，size()-1 改 cardinality()，数组下标改 1 起（ACT-038）；加 SET_VAR(new_planner_optimize_timeout=60000)（DEC-022）；${day}/${hour} 写死为实验窗口 20261001 / 0。</t>
+          <t>UDF 按 DEC-023 原样保留：`default`.format_json_list 包在 unnest 里，default 是保留字所以加反引号；ACT-038 的 parse_json 写法已撤回。库表 default.log_audit_source 改 csc.ods_csc_log_audit（DEC-014）；log_app_id 改 app_id（DEC-015）；sodl 的 day/hour 改 insertdate='2026-10-01' 与 hour(from_unixtime(inserttimestamp))=0（DEC-016/017）；sum(log_num) 改 count(1)（DEC-020）；MANAGE/manage 改 deviceId（DEC-021）；LATERAL VIEW explode(UDF) 改 unnest(UDF)，size()-1 改 cardinality()，数组下标改 1 起；加 SET_VAR(new_planner_optimize_timeout=60000)（DEC-022）；${day}/${hour} 写死为实验窗口 20261001 / 0。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
记录 ACT-054：topthreat_hot_stat UDF 写法执行通过
Co-authored-by: daydayup <removecode@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/业务SQL跑通记录.xlsx
+++ b/outputs/业务SQL跑通记录.xlsx
@@ -645,12 +645,12 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>已跑通（改回UDF后待用户确认）</t>
+          <t>已跑通</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>三条语句此前用户确认已跑通；改回 UDF 写法后待用户确认</t>
+          <t>用户 2026-10-19 确认 UDF 写法也执行通过；详见 ACT-054</t>
         </is>
       </c>
     </row>
@@ -2262,17 +2262,17 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>已跑通（改回UDF后待用户确认）</t>
+          <t>已跑通</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>用户确认已跑通的是 parse_json 写法（2026-10-16）。按 DEC-023 改回 format_json_list 后，只在本机 StarRocks 用 UDF 孪生实现执行过（ACT-046）：黑域名 320 行、黑文件 50 行、黑 URL 620 行，数据为合成数据。用户尚未在当前 StarRocks 确认改回后的语句。</t>
+          <t>用户 2026-10-19 回复“热门威胁也运行通过”，确认 DEC-023 改回 format_json_list 的 UDF 写法在其 StarRocks 执行通过。此前 2026-10-16 已确认 parse_json 写法跑通。执行环境、行数、耗时未提供；本机合成数据结果见 ACT-046、ACT-052。详见 ACT-054</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -2437,17 +2437,17 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>已跑通（改回UDF后待用户确认）</t>
+          <t>已跑通</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>用户确认已跑通的是 parse_json 写法（2026-10-16）。按 DEC-023 改回 format_json_list 后，只在本机 StarRocks 用 UDF 孪生实现执行过（ACT-046）：黑域名 320 行、黑文件 50 行、黑 URL 620 行，数据为合成数据。用户尚未在当前 StarRocks 确认改回后的语句。</t>
+          <t>用户 2026-10-19 回复“热门威胁也运行通过”，确认 DEC-023 改回 format_json_list 的 UDF 写法在其 StarRocks 执行通过。此前 2026-10-16 已确认 parse_json 写法跑通。执行环境、行数、耗时未提供；本机合成数据结果见 ACT-046、ACT-052。详见 ACT-054</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -2623,17 +2623,17 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>已跑通（改回UDF后待用户确认）</t>
+          <t>已跑通</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>用户确认已跑通的是 parse_json 写法（2026-10-16）。按 DEC-023 改回 format_json_list 后，只在本机 StarRocks 用 UDF 孪生实现执行过（ACT-046）：黑域名 320 行、黑文件 50 行、黑 URL 620 行，数据为合成数据。用户尚未在当前 StarRocks 确认改回后的语句。</t>
+          <t>用户 2026-10-19 回复“热门威胁也运行通过”，确认 DEC-023 改回 format_json_list 的 UDF 写法在其 StarRocks 执行通过。此前 2026-10-16 已确认 parse_json 写法跑通。执行环境、行数、耗时未提供；本机合成数据结果见 ACT-046、ACT-052。详见 ACT-054</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">

</xml_diff>